<commit_message>
Completed Phase 4: Built star schema, created dimension tables, configured relationships, and optimized the Power BI data model
</commit_message>
<xml_diff>
--- a/docs/ETL_Process.xlsx
+++ b/docs/ETL_Process.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Samira\Data\Projects\Syntecxhub Internship\1. Week\Sales_Performance_Dashboard\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD4C5FCB-AE1E-49CD-97FD-CDB344B0D32C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{896F4A64-EE39-498B-B422-3C999D71AE4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{4002C09E-2D4E-4A35-B013-734795BD7478}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="92">
   <si>
     <t>Step No.</t>
   </si>
@@ -256,6 +256,51 @@
   </si>
   <si>
     <t>Star Schema</t>
+  </si>
+  <si>
+    <t>Create Reference Tables</t>
+  </si>
+  <si>
+    <t>Created dimension tables (Customer, Product, Category, Geography, Ship Mode, Payment Mode) using Reference queries</t>
+  </si>
+  <si>
+    <t>Dimension Tables</t>
+  </si>
+  <si>
+    <t>Create Date Table</t>
+  </si>
+  <si>
+    <t>Created a dedicated Date dimension for calendar and time-based analysis</t>
+  </si>
+  <si>
+    <t>DimDate</t>
+  </si>
+  <si>
+    <t>Build Star Schema</t>
+  </si>
+  <si>
+    <t>Organized the data model using a star schema with one fact table and multiple dimension tables</t>
+  </si>
+  <si>
+    <t>Power BI Model</t>
+  </si>
+  <si>
+    <t>Create Relationships</t>
+  </si>
+  <si>
+    <t>Created one-to-many relationships between the fact table and all dimension tables</t>
+  </si>
+  <si>
+    <t>Relational Data Model</t>
+  </si>
+  <si>
+    <t>Optimize Data Model</t>
+  </si>
+  <si>
+    <t>Renamed tables, validated data types, organized the model, and prepared it for DAX and reporting</t>
+  </si>
+  <si>
+    <t>Optimized Model</t>
   </si>
 </sst>
 </file>
@@ -313,23 +358,7 @@
   </cellStyles>
   <dxfs count="8">
     <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -350,7 +379,23 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -366,15 +411,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{33CBA8CE-7870-4E84-B279-9824518467F6}" name="الجدول1" displayName="الجدول1" ref="A1:F24" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
-  <autoFilter ref="A1:F24" xr:uid="{33CBA8CE-7870-4E84-B279-9824518467F6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{33CBA8CE-7870-4E84-B279-9824518467F6}" name="الجدول1" displayName="الجدول1" ref="A1:F29" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
+  <autoFilter ref="A1:F29" xr:uid="{33CBA8CE-7870-4E84-B279-9824518467F6}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F29">
+    <sortCondition ref="A1:A29"/>
+  </sortState>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{886EF092-B90D-45F0-8625-398B44CAC095}" name="Step No." dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{A2AEF736-FAA1-4892-882B-55FA0B8170F2}" name="ETL Step" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{7DA6B019-B145-4690-B2FB-051C321F159B}" name="Description" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{4065B1E1-9DD9-44B7-9F2E-059A6A658CB7}" name="Tool" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{329DF123-3CBF-4299-BBA9-187728889ED4}" name="Status" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{931EB7A7-24F9-4A74-9D10-8595ACF43E72}" name="Output" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{886EF092-B90D-45F0-8625-398B44CAC095}" name="Step No." dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{A2AEF736-FAA1-4892-882B-55FA0B8170F2}" name="ETL Step" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{7DA6B019-B145-4690-B2FB-051C321F159B}" name="Description" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{4065B1E1-9DD9-44B7-9F2E-059A6A658CB7}" name="Tool" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{329DF123-3CBF-4299-BBA9-187728889ED4}" name="Status" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{931EB7A7-24F9-4A74-9D10-8595ACF43E72}" name="Output" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -677,7 +725,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F74E5F26-1B54-459B-BDE9-94D04650A162}">
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
@@ -1168,6 +1216,106 @@
         <v>76</v>
       </c>
     </row>
+    <row r="25" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A25" s="2">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A26" s="2">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A27" s="2">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A28" s="2">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A29" s="2">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
updated ETL process tracker
</commit_message>
<xml_diff>
--- a/docs/ETL_Process.xlsx
+++ b/docs/ETL_Process.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Samira\Data\Projects\Syntecxhub Internship\1. Week\Sales_Performance_Dashboard\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{896F4A64-EE39-498B-B422-3C999D71AE4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A2D381E-3922-470F-84CC-19BE7497FE16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{4002C09E-2D4E-4A35-B013-734795BD7478}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{4002C09E-2D4E-4A35-B013-734795BD7478}"/>
   </bookViews>
   <sheets>
     <sheet name="ورقة1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="118">
   <si>
     <t>Step No.</t>
   </si>
@@ -301,6 +301,107 @@
   </si>
   <si>
     <t>Optimized Model</t>
+  </si>
+  <si>
+    <t>Create Measure Table</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Created a dedicated </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Measures</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> table to organize all DAX calculations following Power BI best practices.</t>
+    </r>
+  </si>
+  <si>
+    <t>✅ Completed</t>
+  </si>
+  <si>
+    <t>Measures table</t>
+  </si>
+  <si>
+    <t>Create Base Measures</t>
+  </si>
+  <si>
+    <t>Created reusable DAX measures for Total Revenue, Total Profit, Total Orders, Total Customers, Total Products, Total Quantity Sold, and Returned Orders.</t>
+  </si>
+  <si>
+    <t>DAX</t>
+  </si>
+  <si>
+    <t>Base Measures</t>
+  </si>
+  <si>
+    <t>Create Financial KPIs</t>
+  </si>
+  <si>
+    <t>Built financial measures including Average Order Value, Average Profit per Order, Sales per Customer, Profit per Customer, Orders per Customer, Profit Margin, and Return Rate.</t>
+  </si>
+  <si>
+    <t>Financial KPI Measures</t>
+  </si>
+  <si>
+    <t>Create Time Intelligence Measures</t>
+  </si>
+  <si>
+    <t>Developed time-based measures such as Previous Year Sales, Growth Rate, Sales YTD, and Profit YTD using the Date table.</t>
+  </si>
+  <si>
+    <t>Time Intelligence Measures</t>
+  </si>
+  <si>
+    <t>Create Customer Measures</t>
+  </si>
+  <si>
+    <t>Developed customer analytics measures to evaluate customer value and purchasing behavior.</t>
+  </si>
+  <si>
+    <t>Customer KPI Measures</t>
+  </si>
+  <si>
+    <t>Create Product Measures</t>
+  </si>
+  <si>
+    <t>Developed product performance measures for sales, quantity, profitability, and ranking analysis.</t>
+  </si>
+  <si>
+    <t>Product KPI Measures</t>
+  </si>
+  <si>
+    <t>Create Regional Measures</t>
+  </si>
+  <si>
+    <t>Developed regional performance measures for revenue, profit, and regional comparison.</t>
+  </si>
+  <si>
+    <t>Regional KPI Measures</t>
+  </si>
+  <si>
+    <t>Create Business Measures</t>
+  </si>
+  <si>
+    <t>Developed additional business measures to answer management questions and support dashboard insights.</t>
+  </si>
+  <si>
+    <t>Business Measures</t>
   </si>
 </sst>
 </file>
@@ -411,8 +512,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{33CBA8CE-7870-4E84-B279-9824518467F6}" name="الجدول1" displayName="الجدول1" ref="A1:F29" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
-  <autoFilter ref="A1:F29" xr:uid="{33CBA8CE-7870-4E84-B279-9824518467F6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{33CBA8CE-7870-4E84-B279-9824518467F6}" name="الجدول1" displayName="الجدول1" ref="A1:F37" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
+  <autoFilter ref="A1:F37" xr:uid="{33CBA8CE-7870-4E84-B279-9824518467F6}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F29">
     <sortCondition ref="A1:A29"/>
   </sortState>
@@ -725,18 +826,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F74E5F26-1B54-459B-BDE9-94D04650A162}">
-  <dimension ref="A1:F29"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F37"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" customWidth="1"/>
-    <col min="3" max="3" width="40.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" customWidth="1"/>
+    <col min="3" max="3" width="40.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -756,7 +857,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -776,7 +877,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -796,7 +897,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -816,7 +917,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -836,7 +937,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -856,7 +957,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -876,7 +977,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -896,7 +997,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -916,7 +1017,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -936,7 +1037,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -956,7 +1057,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -976,7 +1077,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -996,7 +1097,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1016,7 +1117,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1036,7 +1137,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1056,7 +1157,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1076,7 +1177,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1096,7 +1197,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1116,7 +1217,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1136,7 +1237,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1156,7 +1257,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1176,7 +1277,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -1196,7 +1297,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -1216,7 +1317,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -1236,7 +1337,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -1256,7 +1357,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -1276,7 +1377,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -1296,7 +1397,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -1314,6 +1415,166 @@
       </c>
       <c r="F29" s="2" t="s">
         <v>91</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A30" s="2">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A31" s="2">
+        <v>5.2</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+      <c r="A32" s="2">
+        <v>5.3</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A33" s="2">
+        <v>5.4</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A34" s="2">
+        <v>5.5</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A35" s="2">
+        <v>5.6</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A36" s="2">
+        <v>5.7</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A37" s="2">
+        <v>5.8</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Completed Phase 6: Dashboard development with interactive pages, drill-through navigation, slicers, KPIs, and updated project documentation
</commit_message>
<xml_diff>
--- a/docs/ETL_Process.xlsx
+++ b/docs/ETL_Process.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Samira\Data\Projects\Syntecxhub Internship\1. Week\Sales_Performance_Dashboard\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A2D381E-3922-470F-84CC-19BE7497FE16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9CFFFED-FBAC-432B-A25F-250B5A2AA128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{4002C09E-2D4E-4A35-B013-734795BD7478}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="153">
   <si>
     <t>Step No.</t>
   </si>
@@ -402,6 +402,111 @@
   </si>
   <si>
     <t>Business Measures</t>
+  </si>
+  <si>
+    <t>Dashboard Planning</t>
+  </si>
+  <si>
+    <t>Designed dashboard layout and navigation</t>
+  </si>
+  <si>
+    <t>Dashboard Design</t>
+  </si>
+  <si>
+    <t>Executive Overview</t>
+  </si>
+  <si>
+    <t>Built executive summary page with KPIs</t>
+  </si>
+  <si>
+    <t>Executive Dashboard</t>
+  </si>
+  <si>
+    <t>Sales Performance</t>
+  </si>
+  <si>
+    <t>Created sales performance dashboard</t>
+  </si>
+  <si>
+    <t>Sales Dashboard</t>
+  </si>
+  <si>
+    <t>Product Analysis</t>
+  </si>
+  <si>
+    <t>Created product performance dashboard</t>
+  </si>
+  <si>
+    <t>Product Dashboard</t>
+  </si>
+  <si>
+    <t>Customer Analysis</t>
+  </si>
+  <si>
+    <t>Built customer analytics page</t>
+  </si>
+  <si>
+    <t>Customer Dashboard</t>
+  </si>
+  <si>
+    <t>Regional Analysis</t>
+  </si>
+  <si>
+    <t>Created regional performance dashboard</t>
+  </si>
+  <si>
+    <t>Regional Dashboard</t>
+  </si>
+  <si>
+    <t>Category Analysis</t>
+  </si>
+  <si>
+    <t>Created category performance page</t>
+  </si>
+  <si>
+    <t>Category Dashboard</t>
+  </si>
+  <si>
+    <t>Return Analysis</t>
+  </si>
+  <si>
+    <t>Developed return analysis visuals</t>
+  </si>
+  <si>
+    <t>Return Dashboard</t>
+  </si>
+  <si>
+    <t>Interactive Slicers</t>
+  </si>
+  <si>
+    <t>Added synchronized report filters</t>
+  </si>
+  <si>
+    <t>Interactive Dashboard</t>
+  </si>
+  <si>
+    <t>Navigation</t>
+  </si>
+  <si>
+    <t>Added page navigation buttons</t>
+  </si>
+  <si>
+    <t>Drill Through</t>
+  </si>
+  <si>
+    <t>Implemented Product Details drill-through page</t>
+  </si>
+  <si>
+    <t>Drill-through Report</t>
+  </si>
+  <si>
+    <t>Dashboard Formatting</t>
+  </si>
+  <si>
+    <t>Applied theme, colors, spacing, titles and icons</t>
+  </si>
+  <si>
+    <t>Professional Dashboard</t>
   </si>
 </sst>
 </file>
@@ -512,8 +617,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{33CBA8CE-7870-4E84-B279-9824518467F6}" name="الجدول1" displayName="الجدول1" ref="A1:F37" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
-  <autoFilter ref="A1:F37" xr:uid="{33CBA8CE-7870-4E84-B279-9824518467F6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{33CBA8CE-7870-4E84-B279-9824518467F6}" name="الجدول1" displayName="الجدول1" ref="A1:F49" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
+  <autoFilter ref="A1:F49" xr:uid="{33CBA8CE-7870-4E84-B279-9824518467F6}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F29">
     <sortCondition ref="A1:A29"/>
   </sortState>
@@ -826,7 +931,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F74E5F26-1B54-459B-BDE9-94D04650A162}">
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" bestFit="1" customWidth="1"/>
@@ -1419,7 +1524,7 @@
     </row>
     <row r="30" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
-        <v>5.0999999999999996</v>
+        <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>92</v>
@@ -1439,7 +1544,7 @@
     </row>
     <row r="31" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
-        <v>5.2</v>
+        <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>96</v>
@@ -1459,7 +1564,7 @@
     </row>
     <row r="32" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
-        <v>5.3</v>
+        <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>100</v>
@@ -1479,7 +1584,7 @@
     </row>
     <row r="33" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
-        <v>5.4</v>
+        <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>103</v>
@@ -1499,7 +1604,7 @@
     </row>
     <row r="34" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
-        <v>5.5</v>
+        <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>106</v>
@@ -1519,7 +1624,7 @@
     </row>
     <row r="35" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
-        <v>5.6</v>
+        <v>34</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>109</v>
@@ -1539,7 +1644,7 @@
     </row>
     <row r="36" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
-        <v>5.7</v>
+        <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>112</v>
@@ -1559,7 +1664,7 @@
     </row>
     <row r="37" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
-        <v>5.8</v>
+        <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>115</v>
@@ -1575,6 +1680,246 @@
       </c>
       <c r="F37" s="2" t="s">
         <v>117</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A38" s="2">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A39" s="2">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A40" s="2">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A41" s="2">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A42" s="2">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A43" s="2">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A44" s="2">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A45" s="2">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A46" s="2">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="2">
+        <v>46</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A48" s="2">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A49" s="2">
+        <v>48</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>152</v>
       </c>
     </row>
   </sheetData>

</xml_diff>